<commit_message>
Bug fix for debit advice ( category dropdown, uplaoding issue when posting , approval in uploading )
</commit_message>
<xml_diff>
--- a/uploads/UPLOAD-TEMPLATE/DEBIT-ADVICE-UPLOAD-TEMPLATE.xlsx
+++ b/uploads/UPLOAD-TEMPLATE/DEBIT-ADVICE-UPLOAD-TEMPLATE.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dvprogio\Desktop\OSH\OSH-APP-Backend\uploads\UPLOAD-TEMPLATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E466777-30F7-4E78-B84E-7BEBF7C51063}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B573180-1679-466D-8274-36F3359B2568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="3900" windowWidth="20730" windowHeight="11040" xr2:uid="{8DE630E0-0B89-4DDE-A92E-DF514EA9A919}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="14">
   <si>
     <t>TEST</t>
   </si>
@@ -64,6 +64,9 @@
   </si>
   <si>
     <t>Damage</t>
+  </si>
+  <si>
+    <t>DOCUMENT REMARKS</t>
   </si>
 </sst>
 </file>
@@ -430,7 +433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAE589B1-C7BA-44D4-9E29-919A5892AA9B}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
@@ -440,9 +443,10 @@
     <col min="5" max="5" width="40.7109375" customWidth="1"/>
     <col min="6" max="6" width="26.7109375" customWidth="1"/>
     <col min="7" max="7" width="37.7109375" customWidth="1"/>
+    <col min="8" max="8" width="21.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
@@ -464,8 +468,11 @@
       <c r="G1" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -487,8 +494,11 @@
       <c r="G2" t="s">
         <v>12</v>
       </c>
+      <c r="H2" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -510,8 +520,11 @@
       <c r="G3" t="s">
         <v>12</v>
       </c>
+      <c r="H3" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -533,8 +546,11 @@
       <c r="G4" t="s">
         <v>12</v>
       </c>
+      <c r="H4" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -556,8 +572,11 @@
       <c r="G5" t="s">
         <v>12</v>
       </c>
+      <c r="H5" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
@@ -577,6 +596,9 @@
         <v>4003</v>
       </c>
       <c r="G6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Additonal location field , added new validation base on location
</commit_message>
<xml_diff>
--- a/uploads/UPLOAD-TEMPLATE/DEBIT-ADVICE-UPLOAD-TEMPLATE.xlsx
+++ b/uploads/UPLOAD-TEMPLATE/DEBIT-ADVICE-UPLOAD-TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dvprogio\Desktop\OSH\OSH-APP-Backend\uploads\UPLOAD-TEMPLATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B573180-1679-466D-8274-36F3359B2568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{108080EC-3937-427B-97CB-67E8D878ADB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="3900" windowWidth="20730" windowHeight="11040" xr2:uid="{8DE630E0-0B89-4DDE-A92E-DF514EA9A919}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8DE630E0-0B89-4DDE-A92E-DF514EA9A919}"/>
   </bookViews>
   <sheets>
     <sheet name="DV" sheetId="1" r:id="rId1"/>
@@ -25,22 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="14">
-  <si>
-    <t>TEST</t>
-  </si>
-  <si>
-    <t>AREA HEAD</t>
-  </si>
-  <si>
-    <t>TEST 2</t>
-  </si>
-  <si>
-    <t>TEST 3</t>
-  </si>
-  <si>
-    <t>TEST 4</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>SEQUENCE</t>
   </si>
@@ -63,10 +48,10 @@
     <t>TRANSACTION DATE</t>
   </si>
   <si>
-    <t>Damage</t>
-  </si>
-  <si>
     <t>DOCUMENT REMARKS</t>
+  </si>
+  <si>
+    <t>LOCATION</t>
   </si>
 </sst>
 </file>
@@ -433,7 +418,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAE589B1-C7BA-44D4-9E29-919A5892AA9B}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
@@ -442,164 +427,78 @@
     <col min="4" max="4" width="36.7109375" customWidth="1"/>
     <col min="5" max="5" width="40.7109375" customWidth="1"/>
     <col min="6" max="6" width="26.7109375" customWidth="1"/>
-    <col min="7" max="7" width="37.7109375" customWidth="1"/>
-    <col min="8" max="8" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.5703125" customWidth="1"/>
+    <col min="8" max="8" width="26.140625" customWidth="1"/>
+    <col min="9" max="9" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>13</v>
-      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" s="2">
         <v>46147</v>
       </c>
-      <c r="C2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>4000</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" t="s">
-        <v>12</v>
-      </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" s="2">
         <v>46147</v>
       </c>
-      <c r="C3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>4001</v>
-      </c>
-      <c r="G3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" t="s">
-        <v>12</v>
-      </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" s="2">
         <v>46147</v>
       </c>
-      <c r="C4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D4" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4" t="s">
-        <v>1</v>
-      </c>
-      <c r="F4">
-        <v>4002</v>
-      </c>
-      <c r="G4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H4" t="s">
-        <v>12</v>
-      </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="B5" s="2">
         <v>46147</v>
       </c>
-      <c r="C5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" t="s">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>4003</v>
-      </c>
-      <c r="G5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H5" t="s">
-        <v>12</v>
-      </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
       <c r="B6" s="2">
         <v>46147</v>
-      </c>
-      <c r="C6" t="s">
-        <v>0</v>
-      </c>
-      <c r="D6" t="s">
-        <v>4</v>
-      </c>
-      <c r="E6" t="s">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>4003</v>
-      </c>
-      <c r="G6" t="s">
-        <v>12</v>
-      </c>
-      <c r="H6" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>